<commit_message>
Update ballParam and add 1 new ball
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B70D5A4-DD5C-4205-A377-E45B698C91CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB0E77D-B4C8-4DD9-9FE4-0F27352BC083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -247,7 +247,7 @@
             <rFont val="Arial"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Leave a fire trail when moving, dealing {Skilldamage} damage to the enemy within</t>
+          <t xml:space="preserve">Leave a fire trail when moving, dealing </t>
         </r>
         <r>
           <rPr>
@@ -257,7 +257,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t xml:space="preserve"> per second</t>
+          <t xml:space="preserve">ball's attack </t>
         </r>
         <r>
           <rPr>
@@ -266,7 +266,69 @@
             <rFont val="Arial"/>
             <scheme val="minor"/>
           </rPr>
-          <t xml:space="preserve">. The trial will last {Skillduration} seconds.
+          <t>damage to the enemy within</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve"> per x second</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">. The trial will last </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">y </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">seconds.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">Variables needed: 
+{LeaveDuration}: float, the duration of the ball leaving the trail, unit in seconds.
+{TrailDuration}: float, the duration of the fire trail, unit in seconds.
+{DamageFrequency}: float, the amount of time required for the trail to calculate damage once, unit in seconds.
+{TrailSize}:  The trail's width, unit in scale. </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">
 </t>
         </r>
       </text>
@@ -280,7 +342,7 @@
             <rFont val="Arial"/>
             <scheme val="minor"/>
           </rPr>
-          <t>The pinball will split into {Skill</t>
+          <t xml:space="preserve">The pinball will split into </t>
         </r>
         <r>
           <rPr>
@@ -290,7 +352,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>effect</t>
+          <t>x</t>
         </r>
         <r>
           <rPr>
@@ -299,7 +361,7 @@
             <rFont val="Arial"/>
             <scheme val="minor"/>
           </rPr>
-          <t xml:space="preserve">} balls, each ball </t>
+          <t xml:space="preserve"> balls, each ball </t>
         </r>
         <r>
           <rPr>
@@ -310,6 +372,9 @@
             <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">cannot be split again further.
+Variables needed:
+{SplitCount}: int, The number of balls that the origin ball split into.
+{SplitSize}: int, The size of the splitted balls, unit in scale.
 </t>
         </r>
       </text>
@@ -323,7 +388,87 @@
             <rFont val="Arial"/>
             <scheme val="minor"/>
           </rPr>
-          <t>When the skill triggers, the ball will shoot out a ring of spikes, dealing {Skilldamage} amount of damage to enemies hit. The spike can travel {Skilldistance}, and ignore terrains.</t>
+          <t xml:space="preserve">When the skill triggers, the ball will shoot out a ring of spikes, dealing </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">ball's attack </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">damage to enemies hit. The spike </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>lasts x seconds as they travel</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>, and ignore terrains.</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve"> (each ring of spikes contains 16 of them(or 8 if optimization becomes an issue)).</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>{SpikeSpeed}: float, the speed of the flying spikes.
+{SpikeSize}: float, the size of the flying spikes.
+{SpikeDuration}: float, the duration of the spike before it disappears.</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Arial"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
         </r>
       </text>
     </comment>
@@ -347,7 +492,10 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Enemies within the area's movement speed will be reduced to zero. The area effect is {Skilleffect}(size multiplier), and the zone lasts{Skillduration}.</t>
+Enemies within the area's movement speed will be reduced to zero. The area effect is x , and the zone lasts y.
+variables needed:
+{ZoneSize}: float, the size of the vfx/area of the icezone, unit in scale.
+{ZoneDuration}: int, the duration of the zone, unit in seconds.</t>
         </r>
       </text>
     </comment>
@@ -371,7 +519,37 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Summons an invisible area surrounding the ball. The area will strike down lightning bolts to enemies contacted, dealing ball's base attack value to them. The area size is {Skilleffect}, and lasts {Skillduration}.</t>
+Summons an invisible area surrounding the ball. The area will strike down lightning bolts to enemies contacted, dealing ball's attack value to them. The area size is x, and lasts y.
+varaibles needed:
+{LightningSize}: float, the detection size of the thunder area, unit in scale.
+{LightningDuration}: float, the duration of the skill.
+{LightningFreq}: float, the cooldown of the thunders on each individual enemies, unit in seconds.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I12" authorId="1" shapeId="0" xr:uid="{18C1C359-D740-41E3-BF5F-1F545E62F512}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Hannya T:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Unleashes a burst from the ball's current location. The burst will stay at the location where's it's triggered, and does not move with the ball. The burst only deal damage once, and disappears as the vfx fades.
+Varaibles needed:
+{CrystalSize}: float, the size of the burst, unit in scale.</t>
         </r>
       </text>
     </comment>
@@ -380,7 +558,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="54">
   <si>
     <t>##var</t>
   </si>
@@ -555,33 +733,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Uses </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Plexus AoE</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> as skill effect vfx.</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>FireTrail</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -622,6 +773,116 @@
   </si>
   <si>
     <t>Drops a fire trail that deals ball's attack damage to enemies within overtime.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Uses </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Crystals crossfade 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> as skill effect vfx.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CrystalBall</t>
+  </si>
+  <si>
+    <t>CrystalBall</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CrystalCrash</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Summons a crystal burst at the ball's current location, dealing ball's attack damage to enemies within.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Attach </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Lightning aura </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>to the ball</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">during skill duraton, and Uses </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Plexus AoE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> as skill effect vfx.</t>
+    </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -945,7 +1206,7 @@
   <cols>
     <col min="11" max="11" width="14.6640625" customWidth="1"/>
     <col min="13" max="13" width="69.33203125" customWidth="1"/>
-    <col min="15" max="15" width="36.21875" customWidth="1"/>
+    <col min="15" max="15" width="38.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1193,7 +1454,7 @@
         <v>500</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J6" s="1">
         <v>250</v>
@@ -1205,13 +1466,13 @@
         <v>25</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
@@ -1249,7 +1510,7 @@
         <v>0.75</v>
       </c>
       <c r="H7" s="1">
-        <v>10000</v>
+        <v>7000</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>19</v>
@@ -1264,7 +1525,7 @@
         <v>27</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>18</v>
@@ -1485,7 +1746,7 @@
         <v>40</v>
       </c>
       <c r="J11" s="1">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="K11" s="1">
         <v>30</v>
@@ -1494,13 +1755,13 @@
         <v>39</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="O11" s="2" t="s">
-        <v>43</v>
+      <c r="O11" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
@@ -1517,22 +1778,48 @@
       <c r="AB11" s="1"/>
       <c r="AC11" s="1"/>
     </row>
-    <row r="12" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
+      <c r="B12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="1">
+        <v>25</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1.25</v>
+      </c>
+      <c r="H12" s="1">
+        <v>500</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J12" s="1">
+        <v>650</v>
+      </c>
+      <c r="K12" s="1">
+        <v>30</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>52</v>
+      </c>
       <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
+      <c r="O12" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>

</xml_diff>

<commit_message>
Adjust spliball size and skill trigger value
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B185303B-3968-4679-881E-7E83030467D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A845CE-BAF4-4098-B5C3-D462411333F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1507,7 +1507,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="1">
-        <v>0.75</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H7" s="1">
         <v>7000</v>

</xml_diff>

<commit_message>
Update skill trigger and damage number font
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A845CE-BAF4-4098-B5C3-D462411333F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA54106-AA6F-46CD-9264-5DCA215A8596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1451,7 +1451,7 @@
         <v>0.8</v>
       </c>
       <c r="H6" s="1">
-        <v>500</v>
+        <v>3500</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>43</v>
@@ -1567,7 +1567,7 @@
         <v>1.35</v>
       </c>
       <c r="H8" s="1">
-        <v>700</v>
+        <v>4000</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>41</v>
@@ -1681,7 +1681,7 @@
         <v>1.25</v>
       </c>
       <c r="H10" s="1">
-        <v>750</v>
+        <v>3000</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>42</v>
@@ -1740,7 +1740,7 @@
         <v>1.1499999999999999</v>
       </c>
       <c r="H11" s="1">
-        <v>900</v>
+        <v>4000</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>40</v>
@@ -1799,7 +1799,7 @@
         <v>1.25</v>
       </c>
       <c r="H12" s="1">
-        <v>500</v>
+        <v>5500</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
Update BallSize and monsterHP
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA54106-AA6F-46CD-9264-5DCA215A8596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1D0388-752B-4AF6-8F2B-EFFCD0526A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1411,7 +1411,7 @@
         <v>1.5</v>
       </c>
       <c r="G5" s="1">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
@@ -1448,7 +1448,7 @@
         <v>2</v>
       </c>
       <c r="G6" s="2">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="H6" s="1">
         <v>3500</v>
@@ -1507,7 +1507,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="1">
-        <v>1.1000000000000001</v>
+        <v>1.05</v>
       </c>
       <c r="H7" s="1">
         <v>7000</v>
@@ -1737,7 +1737,7 @@
         <v>2</v>
       </c>
       <c r="G11" s="1">
-        <v>1.1499999999999999</v>
+        <v>1.25</v>
       </c>
       <c r="H11" s="1">
         <v>4000</v>

</xml_diff>

<commit_message>
Update ball weight value
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CF6A01-29F7-4607-8AC4-EAF846F17019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C72AFE-6009-4EB8-B94C-DE324ECDADFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -558,7 +558,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
   <si>
     <t>##var</t>
   </si>
@@ -621,9 +621,6 @@
   </si>
   <si>
     <t>Spikeball</t>
-  </si>
-  <si>
-    <t>Radiantball</t>
   </si>
   <si>
     <t>float</t>
@@ -1237,13 +1234,13 @@
         <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O1" s="2"/>
       <c r="P1" s="1"/>
@@ -1272,16 +1269,16 @@
         <v>13</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>13</v>
@@ -1296,13 +1293,13 @@
         <v>13</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
@@ -1420,7 +1417,7 @@
         <v>16</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>16</v>
@@ -1450,25 +1447,25 @@
         <v>3500</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J6" s="1">
         <v>250</v>
       </c>
       <c r="K6" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
@@ -1515,13 +1512,13 @@
         <v>400</v>
       </c>
       <c r="K7" s="1">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>18</v>
@@ -1566,7 +1563,7 @@
         <v>4000</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J8" s="1">
         <v>500</v>
@@ -1578,7 +1575,7 @@
         <v>20</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>20</v>
@@ -1602,7 +1599,7 @@
     <row r="9" spans="1:29" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" s="1">
         <v>15</v>
@@ -1627,19 +1624,19 @@
         <v>300</v>
       </c>
       <c r="K9" s="1">
-        <v>60</v>
+        <v>40</v>
       </c>
-      <c r="L9" s="1" t="s">
-        <v>21</v>
+      <c r="L9" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="M9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="O9" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
@@ -1659,7 +1656,7 @@
     <row r="10" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="1">
         <v>13</v>
@@ -1680,25 +1677,25 @@
         <v>3000</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J10" s="1">
         <v>200</v>
       </c>
       <c r="K10" s="1">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
@@ -1718,7 +1715,7 @@
     <row r="11" spans="1:29" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="1">
         <v>17</v>
@@ -1739,7 +1736,7 @@
         <v>4000</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J11" s="1">
         <v>600</v>
@@ -1748,16 +1745,16 @@
         <v>30</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
@@ -1777,7 +1774,7 @@
     <row r="12" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C12" s="1">
         <v>25</v>
@@ -1798,7 +1795,7 @@
         <v>5500</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J12" s="1">
         <v>650</v>
@@ -1807,16 +1804,16 @@
         <v>30</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>

</xml_diff>

<commit_message>
fix stuck problem, increase shelly size, reduce crystal ball chance
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C72AFE-6009-4EB8-B94C-DE324ECDADFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD65FEBE-BE8C-426C-A68F-81D08BAFEFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1801,7 +1801,7 @@
         <v>650</v>
       </c>
       <c r="K12" s="1">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
Update ball material, adjust stenball's name and damage text
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD65FEBE-BE8C-426C-A68F-81D08BAFEFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D82358-F96C-41B1-B4BA-E9B85BDCB449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1627,7 +1627,7 @@
         <v>40</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Lower ball price, update reference
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20D82358-F96C-41B1-B4BA-E9B85BDCB449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0369997-52D1-46BC-81C4-72D4CBD61B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -558,7 +558,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="51">
   <si>
     <t>##var</t>
   </si>
@@ -648,10 +648,6 @@
   </si>
   <si>
     <t>BallIcon</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Stentball</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -1408,7 +1404,7 @@
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K5" s="1">
         <v>80</v>
@@ -1417,7 +1413,7 @@
         <v>16</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>16</v>
@@ -1447,10 +1443,10 @@
         <v>3500</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J6" s="1">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="K6" s="1">
         <v>40</v>
@@ -1459,13 +1455,13 @@
         <v>24</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
@@ -1509,7 +1505,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="1">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="K7" s="1">
         <v>20</v>
@@ -1518,7 +1514,7 @@
         <v>25</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N7" s="1" t="s">
         <v>18</v>
@@ -1563,19 +1559,19 @@
         <v>4000</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J8" s="1">
         <v>500</v>
       </c>
       <c r="K8" s="1">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>20</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>20</v>
@@ -1599,7 +1595,7 @@
     <row r="9" spans="1:29" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C9" s="1">
         <v>15</v>
@@ -1621,22 +1617,22 @@
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="K9" s="1">
         <v>40</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="O9" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
@@ -1656,7 +1652,7 @@
     <row r="10" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C10" s="1">
         <v>13</v>
@@ -1677,7 +1673,7 @@
         <v>3000</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J10" s="1">
         <v>200</v>
@@ -1686,16 +1682,16 @@
         <v>40</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
@@ -1715,7 +1711,7 @@
     <row r="11" spans="1:29" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C11" s="1">
         <v>17</v>
@@ -1736,25 +1732,25 @@
         <v>4000</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J11" s="1">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="K11" s="1">
         <v>30</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O11" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
@@ -1774,7 +1770,7 @@
     <row r="12" spans="1:29" ht="28.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="1">
         <v>25</v>
@@ -1795,7 +1791,7 @@
         <v>5500</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J12" s="1">
         <v>650</v>
@@ -1804,16 +1800,16 @@
         <v>0</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>

</xml_diff>

<commit_message>
Update spikeball and crystalball vfx, adjust level layout, add crystall ball icon
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#BallParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#BallParam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0369997-52D1-46BC-81C4-72D4CBD61B1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67DD02A2-B0F3-440C-84E6-2678721637BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1565,7 +1565,7 @@
         <v>500</v>
       </c>
       <c r="K8" s="1">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>20</v>
@@ -1797,7 +1797,7 @@
         <v>650</v>
       </c>
       <c r="K12" s="1">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>46</v>

</xml_diff>